<commit_message>
Update page content to Go-Live Staff Briefing (1 Feb 2027); add colleague image; new voice clips
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NA4bpYGK5x8Tinj9caZGtd
</commit_message>
<xml_diff>
--- a/docs/Corbit_X_List_Content.xlsx
+++ b/docs/Corbit_X_List_Content.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -648,6 +648,36 @@
         <v>8</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Stuck? Check the guide, ask your champion, log a Command Centre ticket, then update the customer.</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>The bank never asks for a PIN, password or OTP. Never share your login.</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -664,12 +694,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -791,7 +821,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Faster service at the counter, a full 360° view of the customer on one screen, credits and salaries at speed, instant statements for the last 12 months and a more secure account-number format. While we transition, customers are well supported: old account numbers keep working for more than six months after go-live, and cheques with old numbers are accepted for six months.</t>
+          <t>Quicker service at the counter, a 360-degree customer view at the teller point, faster credit and salary processing, statements for the last 12 months straight from Corbit X and a more secure 13-digit account number. While we transition, old account numbers keep working for more than six months after go-live, and cheques with old numbers are accepted until 2 August 2027.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -823,7 +853,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>A few things to know: new account numbers (look them up in Corbit X and share them), cheque and chequebook changes, a short pause in account opening around go-live, and live checks on the Sunday before go-live. Each one has a stop on the journey.</t>
+          <t>A few things to know: new account numbers (look them up in Corbit X and share them), cheque and chequebook changes, a short pause in account opening around go-live, and live checks on Sunday 31 January 2027. Each one has a stop on the journey.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -863,7 +893,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Right here! There are six guides on my journey. Tap 'View Guide' on any stop to see the full poster.</t>
+          <t>Right here! There are six guides on my journey. Tap 'View Guide' on any stop to see the full poster. You will also find guides, staff FAQs and how-to videos on the Corbit X portal on the info portal.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -903,7 +933,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Start with your Branch Operations Supervisor (BOS). For anything else, consult the relevant internal team. Programme support contacts will be listed here.</t>
+          <t>Check the guide or FAQ first, then ask your champion or team lead. If you are still stuck, log a Command Centre ticket with a screenshot, and keep the customer updated while you wait. Contact details for the Command Centre will be listed here.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -935,7 +965,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Yes. Old account numbers will continue to be accepted for more than six months after go-live. The new format keeps the same CIF with “00” added in front. Look up the new number in Corbit X and share it with the customer.</t>
+          <t>Yes. Old account numbers will continue to be accepted for more than six months after go-live. The new account number has 13 digits, and the CIF keeps the same number with “00” added in front. Look up the new number in Corbit X and share it with the customer.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -975,7 +1005,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Account opening pauses during the static data freeze and the first three days after go-live. Start the application in Newgen, receive deposits through the designated GL, and finalise from Thursday after go-live.</t>
+          <t>Account opening pauses during the static data freeze and the first three days after go-live (Monday 1 to Wednesday 3 February). Start the application in Newgen, receive deposits through the designated GL, and finalise from Thursday 4 February.</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1015,7 +1045,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Statements for the last 0–12 months are instant via Corbit X. Older statements (12 months+) come from secure backup, through a cleaner, faster request process.</t>
+          <t>Statements for the last 12 months come straight from Corbit X. Older statements, back to when the account was opened, come from stored backup.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1047,7 +1077,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Cheques with old account numbers are accepted for six months after go-live, subject to the usual checks. Chequebooks recorded more than five years ago won't be migrated, so help those customers find an approved alternative.</t>
+          <t>Cheques with old account numbers are accepted for six months (182 days) after go-live, until 2 August 2027, subject to the usual checks. Chequebooks recorded more than five years ago won't be migrated, so help those customers find an approved alternative. Encourage everyone to reorder early.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1087,7 +1117,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>BOSs open the branch day and all branch staff run live transaction and channel checks with real funds. Don't close the branch day or run end of day on Sunday; continue into Monday.</t>
+          <t>On Sunday 31 January 2027, BOSs open the branch day and all branch staff run live transaction and channel checks with real funds. Don't close the branch day or run end of day on Sunday; continue into Monday and run end of day at close of business.</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1114,6 +1144,110 @@
         <v>11</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>When does Corbit X go live?</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Corbit X goes live on Monday 1 February 2027, in every branch and department at the same time. The final cut-off on the current system is Friday 29 January at 2:00pm.</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>when date go-live golive live start monday february 2027 cut-off</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>See the guide</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>stop:4</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>How do I read the new account number?</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>It has 13 digits. Digits 1 and 2 are the currency (00 cedi, 01 dollar, 02 pound, 03 euro). Digit 3 is the customer type (1 individual, 2 non-individual, 3 banks and others). Digits 4 to 11 are a serial number, and digits 12 and 13 are check digits.</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>account number new 13 digit digits currency customer type format read cif</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>What if someone asks a customer for their OTP?</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>The bank never asks for a PIN, password or OTP, and you must never share your login. Tell the customer, and report anything suspicious to Fraud and Risk.</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>otp pin password fraud scam suspicious login share</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1255,7 +1389,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Account opening pauses briefly, but our welcome never does. Start in Newgen and finalise from Thursday.</t>
+          <t>Account opening pauses briefly, but our welcome never does. Start in Newgen and finalise from Thursday 4 February.</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
@@ -1368,12 +1502,12 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Six Corbit X staff guides are now available</t>
+          <t>Go-live is now Monday 1 February 2027</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Explore them all on Kukua's journey, from account numbers to go-live readiness.</t>
+          <t>Go-live has moved to accommodate other important transactions the Bank is undertaking. The extra weeks help us go live with even greater confidence.</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -1393,12 +1527,12 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Look-up process included in training</t>
+          <t>Six Corbit X staff guides are now available</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Training covers how to find a customer's new account number in Corbit X.</t>
+          <t>Explore them all on Kukua's journey, from account numbers to go-live readiness.</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1418,12 +1552,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Printing new account numbers</t>
+          <t>Look-up process included in training</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Guidance on printing new account numbers for customers will follow.</t>
+          <t>Training covers how to find a customer's new account number in Corbit X.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1664,7 +1798,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2027-02-08T00:00:00+00:00</t>
+          <t>2027-02-01T00:00:00+00:00</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
@@ -1684,7 +1818,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
@@ -1704,7 +1838,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>The Corbit X Staff Guide series is live</t>
+          <t>Go-live is now Monday 1 February 2027</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
@@ -1724,7 +1858,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Six practical guides now cover customer welcomes, account opening during the upgrade, new account numbers, cheques and the Sunday live checks. Read them before your next team huddle.</t>
+          <t>Go-live has moved to accommodate other important transactions the Bank is undertaking. The extra weeks help us go live with even greater confidence. See the new calendar in the timeline below.</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -1744,7 +1878,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
@@ -1764,7 +1898,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
@@ -2056,14 +2190,14 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>During the static data freeze in the week before go-live and the first three days after go-live, account opening is unavailable in Flexcube 11.1 and Corbit X.</t>
+          <t>During the static data freeze in the week before go-live and the first three days after go-live (Monday 1 to Wednesday 3 February 2027), account opening is unavailable in Flexcube 11.1 and Corbit X.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Start | Start in Newgen. Collect all required documents.
 Receive | Receive deposits through the designated GL. Record and monitor every deposit.
-Finalise | Finalise from Thursday after go-live and provide account numbers.</t>
+Finalise | Finalise from Thursday 4 February 2027 and provide account numbers.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -2109,7 +2243,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Old account numbers will continue to be accepted for more than six months after go-live.</t>
+          <t>Old account numbers will continue to be accepted for more than six months after go-live. The new account number has 13 digits, and a customer's CIF gains “00” in front.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -2162,12 +2296,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Accept cheques bearing old account numbers for six months after go-live, subject to the usual checks. After six months, these cheques will no longer be accepted.</t>
+          <t>Accept cheques bearing old account numbers for six months (182 days) after go-live, until 2 August 2027, subject to the usual checks. After that date, these cheques will no longer be accepted.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Accept | Accept old-number cheques for six months after go-live, subject to the usual checks.
+          <t>Accept | Accept old-number cheques until 2 August 2027, subject to the usual checks.
 Encourage | Encourage customers to request new chequebooks early.
 Explain | Explain the transition clearly and help customers with their request.</t>
         </is>
@@ -2260,7 +2394,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>On the Sunday immediately before go-live, BOSs will open the branch day. All branch staff will participate in live transaction and channel checks.</t>
+          <t>On Sunday 31 January 2027, the day before go-live, BOSs will open the branch day. All branch staff will participate in live transaction and channel checks.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -2268,7 +2402,7 @@
           <t>Test | Test deposits, branch transactions, ATMs, the mobile app and other instructed channels.
 Real Funds | These are REAL transactions with REAL funds. Follow controls and report issues promptly.
 Do Not Close | Do not close the branch day or run end of day on Sunday.
-Continue | Continue the same branch day into Monday. Run end of day at the close of business on Monday.</t>
+Continue | Continue the same branch day into Monday 1 February. Run end of day at the close of business on Monday.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -2301,12 +2435,12 @@
   <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
@@ -2356,37 +2490,36 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Awareness</t>
+          <t>Keep your skills sharp</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>megaphone</t>
+          <t>cap</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Now – ongoing</t>
+          <t>26 Oct – 23 Dec 2026</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Building understanding of what Corbit X is, why we are moving and what changes for customers and staff.</t>
+          <t>Regular practice, so everyone is confident on Corbit X before go-live.</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Read the six Corbit X Staff Guides
-Share the key messages in team huddles
-Know where to find answers in the Knowledge Hub</t>
+          <t>Practise twice a week, every week
+Branches: 7:15 – 8:15 am. Departments: one hour, two days a week
+Final session: Wednesday 23 December</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>p | p1
-p | p3
-h | updates
-h | faq</t>
+          <t>h | videos
+h | qrc
+p | p3</t>
         </is>
       </c>
       <c r="G2" s="3" t="n">
@@ -2401,32 +2534,75 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Rest and recharge</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>cap</t>
+          <t>heart</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Before go-live</t>
+          <t>24 Dec 2026 – 3 Jan 2027</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Hands-on learning so every colleague can work confidently in Corbit X, including the new account-number look-up process.</t>
+          <t>A break to celebrate with your loved ones. There are no scheduled sessions.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Complete your assigned training modules
-Practise looking up new account numbers
-Keep the quick reference cards close</t>
+          <t>No scheduled sessions
+Celebrate with your loved ones
+The Corbit X portal stays open if you want a refresher</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>h | faq
+h | videos</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Get go-live ready</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>4 – 22 Jan 2027</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>One hour every working day (15 days): a refresher, then certification for your role.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Branches: 7:15 – 8:15 am. Departments: time set by your HoD
+Complete your refresher, then get certified by 22 January
+Champions check in on your practice; BOSs, BSSMs and HoDs make sure every session happens</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>h | videos
 h | qrc
@@ -2434,50 +2610,6 @@
 p | p2</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Readiness Testing</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Go-live weekend</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Live transaction and channel checks on the Sunday immediately before go-live, led by BOSs with all branch staff participating.</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Test deposits, branch transactions, ATMs and the mobile app
-Real transactions with real funds: follow controls
-Do not close the branch day or run end of day on Sunday</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>p | p6
-h | dates
-h | contacts</t>
-        </is>
-      </c>
       <c r="G4" s="3" t="n">
         <v>3</v>
       </c>
@@ -2490,36 +2622,35 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Go-Live</t>
+          <t>Final systems check</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>rocket</t>
+          <t>chart</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Go-live Monday</t>
+          <t>11 – 17 Jan 2027</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Corbit X opens for business. Continue the same branch day from Sunday and lead every interaction with a warm welcome.</t>
+          <t>Before lift-off, we make sure every record lands safely in Corbit X. Then we fly a full practice mission together on Sunday 17 January.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Run end of day at close of business on Monday
-Start account-opening requests in Newgen
-Smile. Check. Serve.</t>
+          <t>Mon 11 Jan: static data migration
+Wed 13 – Fri 15 Jan: data validation. Sat 16 Jan: financial validation
+Sun 17 Jan: business simulation (migration plus a full day of business replay)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>p | p1
-p | p2
-p | p6</t>
+          <t>h | dates
+h | contacts</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
@@ -2534,82 +2665,82 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Customer Support</t>
+          <t>Lift-off weekend</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
+          <t>rocket</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Fri 29 Jan – Mon 1 Feb 2027</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Friday 29 January is the last day on the current system, with a 2:00pm cut-off. Sunday 31 January is the live-check day. Monday 1 February is go-live.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Fri 29 Jan: finish all transactions by 2:00pm, balance cash and vault, run the final end of day
+Sun 31 Jan: BOSs open the branch day and all staff run live checks with real funds. Do not close the day or run end of day
+Mon 1 Feb: arrive by 7:00am, log in, check printers and apps, welcome every customer and run end of day at close of business</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>p | p6
+p | p1
+h | dates</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>After go-live</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
           <t>heart</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>First weeks after go-live</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Helping customers through the change: new account numbers, cheques, chequebooks and account opening.</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Look up and share new account numbers at every interaction
-Accept old-number cheques subject to the usual checks
-Help customers with affected chequebooks find a way forward</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>p | p3
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>From Mon 1 Feb 2027</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Support for customers and colleagues through the first days, weeks and months.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Mon 1 – Wed 3 Feb: start account openings in Newgen. Accounts are finalised from Thu 4 Feb
+First weeks: hypercare, with daily check-ins, the Command Centre on call and champions on the floor
+Old-number cheques are accepted until 2 August 2027, and old account numbers are still accepted</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>p | p2
+p | p3
 p | p4
 p | p5
 h | contacts</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Stabilization</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>chart</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Six months after go-live</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Embedding new ways of working, closing out transition arrangements and building on the platform.</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Old-number cheques no longer accepted after six months
-Keep encouraging use of new account numbers
-Share feedback to help us improve</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>p | p4
-h | dates
-h | updates
-h | faq</t>
         </is>
       </c>
       <c r="G7" s="3" t="n">
@@ -2941,7 +3072,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Hello! I'm Kukua, your Corbit X guide. Over the coming months, I'll help you discover what Corbit X means for our customers, branches, and teams. Let's get started.</t>
+          <t>Hello! I'm Kukua, your Corbit X guide. Between now and go-live on Monday 1 February 2027, I'll help you discover what Corbit X means for our customers, branches, and teams. Let's get started.</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr"/>
@@ -3067,7 +3198,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Good question! I don't have an answer for that one yet. Try one of the suggested questions, or check with your Branch Operations Supervisor.</t>
+          <t>Good question! I don't have an answer for that one yet. Try one of the suggested questions, or check the guide, ask your champion, and log a Command Centre ticket if you are still stuck.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr"/>
@@ -3091,7 +3222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -3131,17 +3262,17 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Will customers' old account numbers still work after go-live?</t>
+          <t>When does Corbit X go live?</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Yes. Old account numbers will continue to be accepted for more than six months after go-live. Look up the new number in Corbit X using the process covered in training, serve the customer, and share the new number so they use it next time.</t>
+          <t>Corbit X goes live on Monday 1 February 2027, in every branch and department at the same time. The final cut-off on the current system is Friday 29 January at 2:00pm.</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>p3</t>
+          <t>p6</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
@@ -3156,17 +3287,17 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Can customers still use cheques that show their old account number?</t>
+          <t>Will customers' old account numbers still work after go-live?</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Yes, for six months after go-live, subject to the usual checks. After six months these cheques will no longer be accepted, so encourage customers to request new chequebooks early.</t>
+          <t>Yes. Old account numbers will continue to be accepted for more than six months after go-live. The new account number has 13 digits, and the CIF gains “00” in front. Look up the new number in Corbit X using the process covered in training, serve the customer, and share the new number so they use it next time.</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>p4</t>
+          <t>p3</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
@@ -3181,17 +3312,17 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>What about chequebooks recorded more than five years ago?</t>
+          <t>Can customers still use cheques that show their old account number?</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>These chequebooks will not be migrated to Corbit X and can no longer be used. Affected customers have been notified. Explain the position with care, help them access funds through an approved alternative, and assist with a new chequebook where required.</t>
+          <t>Yes, for six months (182 days) after go-live, until 2 August 2027, subject to the usual checks. After that date these cheques will no longer be accepted, so encourage customers to request new chequebooks early.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>p5</t>
+          <t>p4</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
@@ -3206,17 +3337,17 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Can we open new accounts during the upgrade?</t>
+          <t>What about chequebooks recorded more than five years ago?</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Account opening is unavailable in Flexcube 11.1 and Corbit X during the static data freeze (the week before go-live) and for the first three days after go-live. Start the application in Newgen, receive deposits through the designated GL, and finalise from Thursday after go-live. Never turn a customer away.</t>
+          <t>These chequebooks will not be migrated to Corbit X and can no longer be used. Affected customers have been notified. Explain the position with care, help them access funds through an approved alternative, and assist with a new chequebook where required.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>p2</t>
+          <t>p5</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
@@ -3231,17 +3362,17 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>What happens on the Sunday before go-live?</t>
+          <t>Can we open new accounts during the upgrade?</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>BOSs will open the branch day and all branch staff take part in live transaction and channel checks: deposits, branch transactions, ATMs, the mobile app and other instructed channels. These are real transactions with real funds. Do not close the branch day or run end of day on Sunday; continue into Monday and run end of day at close of business.</t>
+          <t>Account opening is unavailable in Flexcube 11.1 and Corbit X during the static data freeze (the week before go-live) and for the first three days after go-live (Monday 1 to Wednesday 3 February). Start the application in Newgen, receive deposits through the designated GL, and finalise from Thursday 4 February. Never turn a customer away.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>p6</t>
+          <t>p2</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
@@ -3256,17 +3387,17 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>What should I do if I'm not sure how to answer a customer?</t>
+          <t>What happens on the Sunday before go-live?</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Pause and check before answering. Consult the relevant internal team, or find the guidebook or procedure in the repository. Never let a system change become a reason to turn a customer away.</t>
+          <t>On Sunday 31 January 2027, BOSs will open the branch day and all branch staff take part in live transaction and channel checks: deposits, branch transactions, ATMs, the mobile app and other instructed channels. These are real transactions with real funds. Do not close the branch day or run end of day on Sunday; continue into Monday and run end of day at close of business.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>p1</t>
+          <t>p6</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
@@ -3281,23 +3412,123 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Will new account numbers be printed for customers?</t>
+          <t>What should I do if I'm not sure how to answer a customer?</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Guidance on printing new account numbers will follow. Until then, look up and share the new number at every interaction.</t>
+          <t>Pause and check before answering. Consult the relevant internal team, or find the guidebook or procedure in the repository. Never let a system change become a reason to turn a customer away.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>p3</t>
+          <t>p1</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
         <v>7</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Will new account numbers be printed for customers?</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Guidance on printing new account numbers will follow. Until then, look up and share the new number at every interaction.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>p3</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>How do I read the new account number?</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>It has 13 digits. Digits 1 and 2 are the currency (00 cedi, 01 dollar, 02 pound, 03 euro). Digit 3 is the customer type (1 individual, 2 non-individual, 3 banks and others). Digits 4 to 11 are a serial number, and digits 12 and 13 are check digits. Always add “00” in front of an existing CIF.</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>p3</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>What should I do if I'm stuck?</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Check the repository guide or FAQ, then ask your champion or team lead. If you are still stuck, log a Command Centre ticket with a screenshot, and update the customer while you wait.</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>p1</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>What if someone asks a customer for their OTP?</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>The bank never asks for a PIN, password or OTP, and you must never share your login. Tell the customer, and report anything suspicious to Fraud and Risk.</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>p1</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3318,7 +3549,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
-    <col width="41" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
@@ -3393,7 +3624,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Start in Newgen, finalise from Thursday</t>
+          <t>Start in Newgen, finalise from Thursday 4 February</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
@@ -3476,7 +3707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -3515,9 +3746,10 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>+ Old numbers accepted for 6+ months
-+ Look up the new number in Corbit X
-+ Share the new number every time</t>
+          <t>+ 13 digits: currency (2), customer type (1), serial (8), check (2)
++ Add “00” before an old CIF
++ Old numbers accepted for more than six months
++ Look up and share the new number every time</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
@@ -3537,7 +3769,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>+ Old-number cheques: 6 months, usual checks
+          <t>+ Old-number cheques: six months (182 days), until 2 August 2027, usual checks
 + Encourage new chequebook requests early
 - Books recorded 5+ years ago can't be used</t>
         </is>
@@ -3561,7 +3793,7 @@
         <is>
           <t>+ Start in Newgen, collect all documents
 + Deposits via the designated GL
-+ Finalise from Thursday after go-live</t>
++ Finalise from Thursday 4 February</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
@@ -3581,9 +3813,10 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>+ Sunday: live checks with real funds
+          <t>+ Fri 29 Jan: finish transactions by the 2:00pm cut-off
++ Sun 31 Jan: live checks with real funds
 - No branch-day close or EOD on Sunday
-+ Run EOD at close of business Monday</t>
++ Mon 1 Feb: arrive by 7:00am; EOD at close of business</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -3605,13 +3838,36 @@
         <is>
           <t>+ Smile &amp; serve. Keep customers informed
 + Listen calmly; pause and check if unsure
-- Never turn a customer away</t>
+- Never turn a customer away
+- Never share your login, PIN or OTP</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>BOS authorisers</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>+ KYC first (STSKYCMN): search by KYC Reference, not by status
++ Then CIF (STSCIF): authorise only after the KYC is done
++ Cheque book request (CASCHBOO): the account must already be open</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3628,7 +3884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -3668,17 +3924,17 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Staff Guide series complete</t>
+          <t>Go-live moves to Monday 1 February 2027</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>All six Corbit X Staff Guide posters are now available in the gallery, covering customer experience, account and chequebook transition, and go-live operations.</t>
+          <t>Go-live has moved to accommodate other important transactions the Bank is undertaking. The extra weeks help us go live with even greater confidence.</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
@@ -3693,7 +3949,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Account-number look-up included in training</t>
+          <t>Staff Guide series complete</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -3703,7 +3959,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Training covers how to look up a customer's new account number in Corbit X. Complete your modules before go-live.</t>
+          <t>All six Corbit X Staff Guide posters are now available in the gallery, covering customer experience, account and chequebook transition, and go-live operations.</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
@@ -3718,7 +3974,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Printing new account numbers</t>
+          <t>Account-number look-up included in training</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -3728,13 +3984,63 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Guidance on printing new account numbers for customers will follow. Watch this space.</t>
+          <t>Training covers how to look up a customer's new account number in Corbit X. Complete your modules before go-live.</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Business simulation 4: 93.4%</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Our overall simulation score rose from 51% to 93.4% across four simulations, 1.6 points from the 95% go-live gate.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Printing new account numbers</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Guidance on printing new account numbers for customers will follow. Watch this space.</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3751,10 +4057,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -3809,23 +4115,23 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Static data freeze begins</t>
+          <t>Static data migration</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Account opening unavailable in Flexcube 11.1 and Corbit X. Start applications in Newgen.</t>
+          <t>Customer and account data moves to Corbit X.</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>-7</v>
+        <v>-21</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Week</t>
+          <t>Day</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -3845,16 +4151,16 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Sunday live checks</t>
+          <t>Data validation begins</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>BOSs open the branch day; all staff run live transaction and channel checks.</t>
+          <t>Every record checked and confirmed, Wednesday 13 to Friday 15 January.</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>-1</v>
+        <v>-19</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>0</v>
@@ -3881,16 +4187,16 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Corbit X go-live</t>
+          <t>Financial validation</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Continue Sunday's branch day; run end of day at close of business.</t>
+          <t>Balances checked to the last pesewa.</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0</v>
+        <v>-16</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>0</v>
@@ -3902,7 +4208,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
@@ -3917,16 +4223,16 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Account opening resumes</t>
+          <t>Business simulation</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Finalise pending applications and provide account numbers.</t>
+          <t>Migration plus a full day of business replay.</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>3</v>
+        <v>-15</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>0</v>
@@ -3938,7 +4244,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
@@ -3953,34 +4259,178 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Old-number cheques end</t>
+          <t>Final cut-off, 2:00pm</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Cheques bearing old account numbers are no longer accepted.</t>
+          <t>Last day on the current system. Balance cash and vault, clear suspense and run the final end of day.</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
+        <v>-3</v>
+      </c>
+      <c r="D6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="3" t="n">
-        <v>6</v>
-      </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Day</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
         <v>5</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Sunday live checks</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>BOSs open the branch day; all staff run live transaction and channel checks. Do not close the day or run end of day.</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Corbit X go-live</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Arrive by 7:00am. Continue Sunday's branch day; run end of day at close of business.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Account opening resumes</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Finalise pending applications and provide account numbers.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Old-number cheques end</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Six months (182 days) after go-live: cheques bearing old account numbers are no longer accepted.</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>182</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4002,8 +4452,8 @@
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="39" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
@@ -4043,7 +4493,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Corbit X Programme Office</t>
+          <t>Your champion</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -4053,12 +4503,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Programme questions and feedback</t>
+          <t>First line of help: local support and floor-walking</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>[Add email / extension]</t>
+          <t>[Add name]</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -4073,17 +4523,17 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Branch Operations Support</t>
+          <t>Command Centre</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>shield</t>
+          <t>phoneapp</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Go-live weekend and branch-day issues</t>
+          <t>Log a ticket with a screenshot: issues, fixes and coordination</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -4103,17 +4553,17 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>IT Service Desk</t>
+          <t>Branch Operations Support</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>phoneapp</t>
+          <t>shield</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>System access and technical faults</t>
+          <t>Go-live weekend and branch-day issues</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -4193,7 +4643,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Your Regional Champion</t>
+          <t>Fraud and Risk</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -4203,12 +4653,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Local support and floor-walking</t>
+          <t>Report anything suspicious. The bank never asks for a PIN, password or OTP</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>[Add name]</t>
+          <t>[Add contact]</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -4231,7 +4681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -4274,7 +4724,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Smile. Check. Serve.</t>
+          <t>Same warm welcome. New system. One team.</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
@@ -4289,7 +4739,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Look it up. Share it. Keep banking moving.</t>
+          <t>Smile. Check. Serve.</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
@@ -4304,7 +4754,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Check together. Start strong.</t>
+          <t>Look it up. Share it. Keep banking moving.</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -4319,7 +4769,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Give customers a head start!</t>
+          <t>Check together. Start strong.</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
@@ -4334,13 +4784,43 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Here for your journey</t>
+          <t>Never turn a customer away.</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Give customers a head start!</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Here for your journey</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4396,7 +4876,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Look how far we've come together! These numbers show the energy our people are putting into Corbit X.</t>
+          <t>Look how far we've come together! Our simulation score rose from 51% to 93.4%, and confidence has nearly doubled.</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
@@ -4476,7 +4956,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>So, what's next? Here are the steps that will take us from today all the way to go-live.</t>
+          <t>So, what's next? Here are the five steps that take us from today to go-live on Monday 1 February 2027.</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
@@ -4617,7 +5097,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Old account numbers will continue to be accepted for more than six months after go-live.</t>
+          <t>Old account numbers will continue to be accepted for more than six months after go-live. The new account number has 13 digits, and a customer's CIF gains “00” in front.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -4680,12 +5160,12 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Cheques bearing old account numbers are accepted for six months after go-live, subject to the usual checks. After six months, these cheques will no longer be accepted.</t>
+          <t>Cheques bearing old account numbers are accepted for six months (182 days) after go-live, until 2 August 2027, subject to the usual checks. After that date, these cheques will no longer be accepted.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Accept | Accept old-number cheques for six months after go-live, subject to the usual checks.
+          <t>Accept | Accept old-number cheques until 2 August 2027, subject to the usual checks.
 Encourage | Encourage customers to request new chequebooks early.
 Explain | Explain the transition clearly and help customers with their request.</t>
         </is>
@@ -4798,15 +5278,16 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>On the Sunday immediately before go-live, BOSs will open the branch day. All branch staff will take part in live transaction and channel checks.</t>
+          <t>On Sunday 31 January 2027, the day before go-live, BOSs will open the branch day. All branch staff will take part in live transaction and channel checks.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Test | Test deposits, branch transactions, ATMs, the mobile app and other instructed channels.
+          <t>Friday 29 January | Finish all transactions by the 2:00pm cut-off, balance cash and vault, clear suspense and run the final end of day.
+Test | On Sunday, test deposits, branch transactions, ATMs, the mobile app and other instructed channels.
 Real funds | These are real transactions with real funds. Follow controls and report issues promptly.
 Don't close | Do not close the branch day or run end of day on Sunday.
-Continue | Continue the same branch day into Monday. Run end of day at the close of business on Monday.</t>
+Continue | Continue the same branch day into Monday 1 February. Run end of day at the close of business on Monday.</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr"/>
@@ -4918,14 +5399,14 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>During the static data freeze in the week before go-live and the first three days after go-live, account opening is unavailable in Flexcube 11.1 and Corbit X.</t>
+          <t>During the static data freeze in the week before go-live and the first three days after go-live (Monday 1 to Wednesday 3 February), account opening is unavailable in Flexcube 11.1 and Corbit X.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Start | Start in Newgen. Collect all required documents.
 Receive | Receive deposits through the designated GL. Record and monitor every deposit.
-Finalise | Finalise from Thursday after go-live and provide account numbers.</t>
+Finalise | Finalise from Thursday 4 February and provide account numbers.</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -4962,8 +5443,8 @@
   <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="54" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -5017,30 +5498,30 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Staff bank-wide</t>
+          <t>Overall simulation score (95% go-live gate)</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>No. of Staff</t>
+          <t>Overall readiness</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2500</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G2" s="3" t="n">
@@ -5055,21 +5536,21 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Project completion rate</t>
+          <t>Staff confident in go-live readiness (45% at BSIM 1)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>No. of Staff</t>
+          <t>Overall readiness</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
@@ -5093,25 +5574,25 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Champions across the bank</t>
+          <t>Logged in at BSIM 4</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Staff Engagement</t>
+          <t>System and support</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>heart</t>
+          <t>check</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>30</v>
+        <v>99.8</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -5131,23 +5612,27 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Bank-wide roadshows</t>
+          <t>Tickets fixed the same day</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Staff Engagement</t>
+          <t>System and support</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>heart</t>
+          <t>check</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" s="3" t="inlineStr"/>
+        <v>96</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -5165,23 +5650,27 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Business simulations</t>
+          <t>Branches ready</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Business Simulation</t>
+          <t>Branches</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>users</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" s="3" t="inlineStr"/>
+        <v>94</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -5199,30 +5688,26 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Staff confidence</t>
+          <t>Business simulations completed</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Business Simulation</t>
+          <t>Branches</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>users</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>68</v>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G7" s="3" t="n">
@@ -5296,9 +5781,9 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Serve customers faster
-Full 360° view in one screen
-Credits and salaries at speed</t>
+          <t>Quicker service at the counter
+360-degree customer view at the teller point
+Faster credit and salary processing</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -5328,9 +5813,9 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>New format, same CIF: add “00” in front
-Old numbers usable during the transition
-Longer format = more security</t>
+          <t>New 13-digit account numbers
+Customer CIF gains “00” in front
+Old numbers still work for more than six months</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -5360,9 +5845,9 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Order new books within 182 days
-Current leaves accepted meanwhile
-Books 5+ years old won't migrate</t>
+          <t>Reorder within the first 182 days
+Current leaves accepted in the meantime
+Books over 5 years old are not migrated</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -5392,9 +5877,8 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>0–12 months: instant via Corbit X
-12 months+: from secure backup
-Cleaner, faster request process</t>
+          <t>0–12 months: straight from Corbit X
+Older statements, back to account opening: from stored backup</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -5632,7 +6116,7 @@
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="43" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -5761,7 +6245,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Start in Newgen, finalise from Thursday</t>
+          <t>Start in Newgen, finalise from Thursday 4 February</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr"/>
@@ -5919,7 +6403,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -5961,17 +6445,17 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Complete your training</t>
+          <t>Keep your skills sharp</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Keep learning</t>
+          <t>26 Oct – 23 Dec</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Finish your end-user training modules and practise the new processes.</t>
+          <t>Practise twice a week. Branches 7:15 – 8:15 am; departments one hour, two days a week.</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -5991,22 +6475,22 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Business simulations</t>
+          <t>Rest and recharge</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Practise</t>
+          <t>24 Dec – 3 Jan</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Take part in simulations to build confidence before go-live.</t>
+          <t>No scheduled sessions. The Corbit X portal stays open if you want a refresher.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>heart</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -6021,22 +6505,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Meet your champion</t>
+          <t>Get go-live ready</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Connect</t>
+          <t>4 – 22 Jan</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Our 30+ Corbit X champions are on hand to answer questions locally.</t>
+          <t>One hour every working day, then certification for your role.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>check</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -6051,22 +6535,22 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Sunday live checks</t>
+          <t>Final systems check</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Get ready</t>
+          <t>11 – 17 Jan</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Join the live transaction and channel checks on the Sunday before go-live.</t>
+          <t>Data migration and validation, then the business simulation on Sunday 17 January.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -6081,17 +6565,17 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Same warm welcome</t>
+          <t>Lift-off!</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Go-live</t>
+          <t>Mon 1 Feb 2027</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Serve every customer with confidence on Corbit X.</t>
+          <t>Corbit X goes live. Arrive early, log in and welcome every customer.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">

</xml_diff>